<commit_message>
docs(growth): membership pricing model — ₪6/mo, first vote then free
Replaces per-vote ₪5 with a monthly membership: first vote of a calendar
month costs ₪6, rest free. ₪6 splits ₪2.10 -> monthly civic pool / ₪3.90
platform (net +₪2.47/member/mo). Treasury is now a monthly pool allocated
to executed decisions, not a per-vote credit. Rebuilds the financial model
(Target ~8k members + 900 creates -> ₪40k take-home), PRD, bags spec,
roadmap, and the war-room dashboard incl. the break-even calculator.
</commit_message>
<xml_diff>
--- a/growth/financial-model.xlsx
+++ b/growth/financial-model.xlsx
@@ -8,9 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-even" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,15 +38,8 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00E0301E"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +49,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0014110E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0301E"/>
       </patternFill>
     </fill>
     <fill>
@@ -83,17 +69,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,12 +442,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,7 +460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Locked 2026-06-24 · all figures ₪ unless noted · rate USD/ILS=3.70</t>
+          <t>Updated 2026-06-29 · ₪ · MEMBERSHIP model (first vote/month ₪6, rest free)</t>
         </is>
       </c>
     </row>
@@ -502,171 +485,182 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>USD/ILS rate</t>
+          <t>Member fee / month</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.7</v>
+        <v>6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>assumption, early 2026</t>
+          <t>first vote of the calendar month; rest free</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Paddle fee %</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
+          <t>→ Treasury share</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Merchant-of-Record</t>
+          <t>to monthly civic pool / member</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Paddle fixed / txn</t>
+          <t>→ Platform share</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.85</v>
+        <v>3.9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$0.50</t>
+          <t>before GI fee</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Vote gross</t>
+          <t>GI fee on ₪6</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>1.43</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>participation fee</t>
+          <t>1.4% + ₪1.2 + ₪0.15 receipt</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Platform skim</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
+          <t>Platform NET / member / mo</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.47</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>of each participation</t>
+          <t>after GI fee</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Treasury share</t>
+          <t>Create gross / NET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>50.0 / 47.95</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>funds the civic decision</t>
+          <t>100% platform</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Create gross</t>
+          <t>Avg votes / member / mo</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100% to platform</t>
+          <t>assumption — funnel context only</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fixed costs / mo</t>
+          <t>GI plan / mo</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1200</v>
+        <v>155</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>infra + tooling</t>
+          <t>Prime</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Combined take-home target</t>
+          <t>Fixed costs / mo</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>37500</v>
+        <v>1355</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>midpoint of ₪30–45k</t>
+          <t>infra + tooling + GI Prime</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Effective tax+BL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>27%</t>
-        </is>
+          <t>Take-home target</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>37500</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2x osek murshe est.</t>
+          <t>midpoint ₪30–45k</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>→ Gross-profit target / mo</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>52570</v>
+          <t>Effective tax+BL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
+        <is>
+          <t>2x osek murshe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>→ Gross-profit target</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>52725</v>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>to net the take-home</t>
         </is>
@@ -683,23 +677,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>PARTICIPATION — single charge vs wallet packs</t>
+          <t>MONTHLY SCENARIOS (membership + create-led)</t>
         </is>
       </c>
     </row>
@@ -707,328 +706,67 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Pack ₪</t>
+          <t>Scenario</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Votes</t>
+          <t>Ambassadors</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Paddle fee</t>
+          <t>Paying members</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Skim 30%</t>
+          <t>Votes (ctx)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Platform NET</t>
+          <t>Paid creates</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Platform/vote</t>
+          <t>Member rev</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Create rev</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Treasury/vote</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>30</v>
-      </c>
-      <c r="B5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C5" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="D5" t="n">
-        <v>9</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="G5" t="n">
-        <v>21</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>60</v>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" t="n">
-        <v>4.85</v>
-      </c>
-      <c r="D6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E6" t="n">
-        <v>13.15</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.657</v>
-      </c>
-      <c r="G6" t="n">
-        <v>42</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>150</v>
-      </c>
-      <c r="B7" t="n">
-        <v>50</v>
-      </c>
-      <c r="C7" t="n">
-        <v>9.35</v>
-      </c>
-      <c r="D7" t="n">
-        <v>45</v>
-      </c>
-      <c r="E7" t="n">
-        <v>35.65</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.713</v>
-      </c>
-      <c r="G7" t="n">
-        <v>105</v>
-      </c>
-      <c r="H7" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>300</v>
-      </c>
-      <c r="B8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" t="n">
-        <v>16.85</v>
-      </c>
-      <c r="D8" t="n">
-        <v>90</v>
-      </c>
-      <c r="E8" t="n">
-        <v>73.15000000000001</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.732</v>
-      </c>
-      <c r="G8" t="n">
-        <v>210</v>
-      </c>
-      <c r="H8" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>↑ ₪3 single charge loses money — platform NET negative. Wallet packs fix it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>CREATE VOTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Gross</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Paddle fee</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Platform NET</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Treasury</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>50</v>
-      </c>
-      <c r="B14" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="C14" t="n">
-        <v>45.65</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>MONTHLY SCENARIOS (create-led P&amp;L)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Ambassadors</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Paid creates/mo</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Funded creates</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Total creates</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Part./create</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Participations</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Rev creates</t>
+          <t>Treasury ops</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Rev part.</t>
+          <t>Gross rev</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Gross rev</t>
+          <t>Costs</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Costs</t>
+          <t>Gross profit</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Gross profit</t>
+          <t>Take-home</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Est. take-home</t>
+          <t>Civic pool</t>
         </is>
       </c>
     </row>
@@ -1042,37 +780,37 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>250</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>2000</v>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F4" t="n">
-        <v>30</v>
+        <v>616</v>
       </c>
       <c r="G4" t="n">
-        <v>990</v>
+        <v>1438</v>
       </c>
       <c r="H4" t="n">
-        <v>1141</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>650</v>
+        <v>2055</v>
       </c>
       <c r="J4" t="n">
-        <v>1792</v>
+        <v>1555</v>
       </c>
       <c r="K4" t="n">
-        <v>1400</v>
+        <v>500</v>
       </c>
       <c r="L4" t="n">
-        <v>392</v>
+        <v>365</v>
       </c>
       <c r="M4" t="n">
-        <v>286</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5">
@@ -1085,80 +823,80 @@
         <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>120</v>
+        <v>1500</v>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>12000</v>
       </c>
       <c r="E5" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>3699</v>
       </c>
       <c r="G5" t="n">
-        <v>5600</v>
+        <v>7192</v>
       </c>
       <c r="H5" t="n">
-        <v>5478</v>
+        <v>2500</v>
       </c>
       <c r="I5" t="n">
-        <v>3679</v>
+        <v>10892</v>
       </c>
       <c r="J5" t="n">
-        <v>9157</v>
+        <v>4355</v>
       </c>
       <c r="K5" t="n">
-        <v>1700</v>
+        <v>6536</v>
       </c>
       <c r="L5" t="n">
-        <v>7457</v>
+        <v>4772</v>
       </c>
       <c r="M5" t="n">
-        <v>5444</v>
+        <v>3150</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Target (living)</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>650</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>32500</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>27390</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>21352</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>48742</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>46342</v>
-      </c>
-      <c r="M6" s="7" t="n">
-        <v>33830</v>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Target (band)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>64000</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>19728</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>43155</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>62883</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>7555</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>55328</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>40389</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>16800</v>
       </c>
     </row>
     <row r="7">
@@ -1168,174 +906,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C7" t="n">
-        <v>1800</v>
+        <v>30000</v>
       </c>
       <c r="D7" t="n">
-        <v>120</v>
+        <v>240000</v>
       </c>
       <c r="E7" t="n">
-        <v>1920</v>
+        <v>3000</v>
       </c>
       <c r="F7" t="n">
-        <v>70</v>
+        <v>73980</v>
       </c>
       <c r="G7" t="n">
-        <v>134400</v>
+        <v>143850</v>
       </c>
       <c r="H7" t="n">
-        <v>82170</v>
+        <v>8000</v>
       </c>
       <c r="I7" t="n">
-        <v>88301</v>
+        <v>217830</v>
       </c>
       <c r="J7" t="n">
-        <v>170471</v>
+        <v>11855</v>
       </c>
       <c r="K7" t="n">
-        <v>3700</v>
+        <v>205975</v>
       </c>
       <c r="L7" t="n">
-        <v>166771</v>
+        <v>150362</v>
       </c>
       <c r="M7" t="n">
-        <v>121743</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>BREAK-EVEN (creates-only lens)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Create NET (after Paddle)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>45.65</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>₪ per paid create</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cover fixed costs</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>paid creates/mo (zero salary)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  = per day</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>creates/day</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Hit gross-profit target</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1152</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>paid creates/mo for ₪52570 GP</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  = per day</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>38</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>creates/day</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Participation-only alt.</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>80015</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>paid votes/mo if creates=0 (unrealistic)</t>
-        </is>
+        <v>63000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>